<commit_message>
testing sheet final 2.0
</commit_message>
<xml_diff>
--- a/Testing sheet FINAL.xlsx
+++ b/Testing sheet FINAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b0a90a88555305b7/Desktop/New folder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b0a90a88555305b7/Desktop/algonest/AlgoNest/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D8468B5-B0BA-454A-AF6D-8847F3FDDCCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{1D8468B5-B0BA-454A-AF6D-8847F3FDDCCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05E39059-5C75-42CF-884A-D63ABA70186D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="236">
   <si>
     <t>Sr.No</t>
   </si>
@@ -683,9 +683,6 @@
     <t>bug_02</t>
   </si>
   <si>
-    <t>bug_03</t>
-  </si>
-  <si>
     <t>bug_04</t>
   </si>
   <si>
@@ -798,6 +795,9 @@
   </si>
   <si>
     <t>sc_01G12E2A2:G15A2:H17E2A2:G15A2:I17A2:I17</t>
+  </si>
+  <si>
+    <t>error must be shown ( phone number is invalid )</t>
   </si>
 </sst>
 </file>
@@ -1209,6 +1209,9 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1229,9 +1232,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1522,10 +1522,10 @@
       <c r="A2" s="21">
         <v>1</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="49" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="14" t="s">
@@ -1574,8 +1574,8 @@
       <c r="A3" s="21">
         <v>2</v>
       </c>
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
       <c r="D3" s="14" t="s">
         <v>18</v>
       </c>
@@ -1622,8 +1622,8 @@
       <c r="A4" s="24">
         <v>3</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
       <c r="D4" s="14" t="s">
         <v>43</v>
       </c>
@@ -1670,8 +1670,8 @@
       <c r="A5" s="21">
         <v>4</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
+      <c r="B5" s="50"/>
+      <c r="C5" s="50"/>
       <c r="D5" s="16" t="s">
         <v>48</v>
       </c>
@@ -1718,8 +1718,8 @@
       <c r="A6" s="21">
         <v>5</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
+      <c r="B6" s="50"/>
+      <c r="C6" s="50"/>
       <c r="D6" s="24" t="s">
         <v>55</v>
       </c>
@@ -1766,8 +1766,8 @@
       <c r="A7" s="21">
         <v>6</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
       <c r="D7" s="24" t="s">
         <v>56</v>
       </c>
@@ -1814,8 +1814,8 @@
       <c r="A8" s="24">
         <v>7</v>
       </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="49"/>
+      <c r="B8" s="50"/>
+      <c r="C8" s="50"/>
       <c r="D8" s="24" t="s">
         <v>59</v>
       </c>
@@ -1862,8 +1862,8 @@
       <c r="A9" s="21">
         <v>8</v>
       </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50"/>
       <c r="D9" s="24" t="s">
         <v>62</v>
       </c>
@@ -1910,8 +1910,8 @@
       <c r="A10" s="21">
         <v>9</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="49"/>
+      <c r="B10" s="50"/>
+      <c r="C10" s="50"/>
       <c r="D10" s="24" t="s">
         <v>87</v>
       </c>
@@ -1958,8 +1958,8 @@
       <c r="A11" s="21">
         <v>10</v>
       </c>
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
+      <c r="B11" s="51"/>
+      <c r="C11" s="51"/>
       <c r="D11" s="27" t="s">
         <v>95</v>
       </c>
@@ -2006,10 +2006,10 @@
       <c r="A12" s="24">
         <v>11</v>
       </c>
-      <c r="B12" s="51" t="s">
+      <c r="B12" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="49" t="s">
         <v>67</v>
       </c>
       <c r="D12" s="27" t="s">
@@ -2058,8 +2058,8 @@
       <c r="A13" s="21">
         <v>12</v>
       </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="49"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="50"/>
       <c r="D13" s="27" t="s">
         <v>18</v>
       </c>
@@ -2106,8 +2106,8 @@
       <c r="A14" s="21">
         <v>13</v>
       </c>
-      <c r="B14" s="52"/>
-      <c r="C14" s="49"/>
+      <c r="B14" s="53"/>
+      <c r="C14" s="50"/>
       <c r="D14" s="27" t="s">
         <v>43</v>
       </c>
@@ -2154,8 +2154,8 @@
       <c r="A15" s="21">
         <v>14</v>
       </c>
-      <c r="B15" s="52"/>
-      <c r="C15" s="49"/>
+      <c r="B15" s="53"/>
+      <c r="C15" s="50"/>
       <c r="D15" s="27" t="s">
         <v>48</v>
       </c>
@@ -2202,8 +2202,8 @@
       <c r="A16" s="24">
         <v>15</v>
       </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="49"/>
+      <c r="B16" s="53"/>
+      <c r="C16" s="50"/>
       <c r="D16" s="27" t="s">
         <v>55</v>
       </c>
@@ -2250,8 +2250,8 @@
       <c r="A17" s="21">
         <v>16</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="49"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="50"/>
       <c r="D17" s="27" t="s">
         <v>18</v>
       </c>
@@ -2298,8 +2298,8 @@
       <c r="A18" s="21">
         <v>17</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="49"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="50"/>
       <c r="D18" s="27" t="s">
         <v>43</v>
       </c>
@@ -2346,8 +2346,8 @@
       <c r="A19" s="21">
         <v>18</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="49"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="50"/>
       <c r="D19" s="27" t="s">
         <v>48</v>
       </c>
@@ -2394,8 +2394,8 @@
       <c r="A20" s="24">
         <v>19</v>
       </c>
-      <c r="B20" s="52"/>
-      <c r="C20" s="49"/>
+      <c r="B20" s="53"/>
+      <c r="C20" s="50"/>
       <c r="D20" s="27" t="s">
         <v>55</v>
       </c>
@@ -2442,8 +2442,8 @@
       <c r="A21" s="21">
         <v>20</v>
       </c>
-      <c r="B21" s="52"/>
-      <c r="C21" s="49"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="50"/>
       <c r="D21" s="27" t="s">
         <v>56</v>
       </c>
@@ -2490,8 +2490,8 @@
       <c r="A22" s="21">
         <v>21</v>
       </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="49"/>
+      <c r="B22" s="53"/>
+      <c r="C22" s="50"/>
       <c r="D22" s="27" t="s">
         <v>59</v>
       </c>
@@ -2538,8 +2538,8 @@
       <c r="A23" s="21">
         <v>22</v>
       </c>
-      <c r="B23" s="52"/>
-      <c r="C23" s="49"/>
+      <c r="B23" s="53"/>
+      <c r="C23" s="50"/>
       <c r="D23" s="27" t="s">
         <v>62</v>
       </c>
@@ -2586,8 +2586,8 @@
       <c r="A24" s="24">
         <v>23</v>
       </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="49"/>
+      <c r="B24" s="53"/>
+      <c r="C24" s="50"/>
       <c r="D24" s="27" t="s">
         <v>87</v>
       </c>
@@ -2634,8 +2634,8 @@
       <c r="A25" s="21">
         <v>24</v>
       </c>
-      <c r="B25" s="52"/>
-      <c r="C25" s="49"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="50"/>
       <c r="D25" s="27" t="s">
         <v>95</v>
       </c>
@@ -2682,8 +2682,8 @@
       <c r="A26" s="21">
         <v>25</v>
       </c>
-      <c r="B26" s="52"/>
-      <c r="C26" s="49"/>
+      <c r="B26" s="53"/>
+      <c r="C26" s="50"/>
       <c r="D26" s="27" t="s">
         <v>101</v>
       </c>
@@ -2730,8 +2730,8 @@
       <c r="A27" s="21">
         <v>26</v>
       </c>
-      <c r="B27" s="52"/>
-      <c r="C27" s="49"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="50"/>
       <c r="D27" s="27" t="s">
         <v>105</v>
       </c>
@@ -2778,8 +2778,8 @@
       <c r="A28" s="24">
         <v>27</v>
       </c>
-      <c r="B28" s="52"/>
-      <c r="C28" s="49"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="50"/>
       <c r="D28" s="27" t="s">
         <v>108</v>
       </c>
@@ -2826,8 +2826,8 @@
       <c r="A29" s="21">
         <v>28</v>
       </c>
-      <c r="B29" s="52"/>
-      <c r="C29" s="49"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="50"/>
       <c r="D29" s="27" t="s">
         <v>112</v>
       </c>
@@ -2874,8 +2874,8 @@
       <c r="A30" s="21">
         <v>29</v>
       </c>
-      <c r="B30" s="52"/>
-      <c r="C30" s="49"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="50"/>
       <c r="D30" s="27" t="s">
         <v>180</v>
       </c>
@@ -2922,8 +2922,8 @@
       <c r="A31" s="21">
         <v>30</v>
       </c>
-      <c r="B31" s="52"/>
-      <c r="C31" s="49"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="50"/>
       <c r="D31" s="27" t="s">
         <v>181</v>
       </c>
@@ -2970,8 +2970,8 @@
       <c r="A32" s="24">
         <v>31</v>
       </c>
-      <c r="B32" s="52"/>
-      <c r="C32" s="49"/>
+      <c r="B32" s="53"/>
+      <c r="C32" s="50"/>
       <c r="D32" s="27" t="s">
         <v>182</v>
       </c>
@@ -3018,8 +3018,8 @@
       <c r="A33" s="21">
         <v>32</v>
       </c>
-      <c r="B33" s="52"/>
-      <c r="C33" s="49"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="50"/>
       <c r="D33" s="27" t="s">
         <v>183</v>
       </c>
@@ -3066,8 +3066,8 @@
       <c r="A34" s="21">
         <v>33</v>
       </c>
-      <c r="B34" s="52"/>
-      <c r="C34" s="49"/>
+      <c r="B34" s="53"/>
+      <c r="C34" s="50"/>
       <c r="D34" s="27" t="s">
         <v>184</v>
       </c>
@@ -3114,8 +3114,8 @@
       <c r="A35" s="21">
         <v>34</v>
       </c>
-      <c r="B35" s="52"/>
-      <c r="C35" s="49"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="50"/>
       <c r="D35" s="27" t="s">
         <v>185</v>
       </c>
@@ -3162,8 +3162,8 @@
       <c r="A36" s="24">
         <v>35</v>
       </c>
-      <c r="B36" s="52"/>
-      <c r="C36" s="49"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="50"/>
       <c r="D36" s="27" t="s">
         <v>186</v>
       </c>
@@ -3210,10 +3210,10 @@
       <c r="A37" s="21">
         <v>36</v>
       </c>
-      <c r="B37" s="46" t="s">
+      <c r="B37" s="47" t="s">
         <v>119</v>
       </c>
-      <c r="C37" s="47" t="s">
+      <c r="C37" s="48" t="s">
         <v>113</v>
       </c>
       <c r="D37" s="34" t="s">
@@ -3262,8 +3262,8 @@
       <c r="A38" s="21">
         <v>37</v>
       </c>
-      <c r="B38" s="46"/>
-      <c r="C38" s="47"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="48"/>
       <c r="D38" s="30" t="s">
         <v>18</v>
       </c>
@@ -10878,7 +10878,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1000"/>
+  <dimension ref="A1:AA999"/>
   <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.77734375" customWidth="1"/>
@@ -10952,41 +10952,41 @@
       <c r="AA1" s="12"/>
     </row>
     <row r="2" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="53" t="s">
-        <v>235</v>
-      </c>
-      <c r="B2" s="53" t="s">
+      <c r="A2" s="46" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="53" t="s">
-        <v>234</v>
-      </c>
-      <c r="F2" s="53" t="s">
+      <c r="E2" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="F2" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="53" t="s">
+      <c r="G2" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="53" t="s">
+      <c r="H2" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53" t="s">
+      <c r="I2" s="46"/>
+      <c r="J2" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K2" s="53" t="s">
+      <c r="K2" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="53" t="s">
+      <c r="L2" s="46" t="s">
         <v>187</v>
       </c>
-      <c r="M2" s="53" t="s">
+      <c r="M2" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O2" s="12"/>
@@ -11004,41 +11004,41 @@
       <c r="AA2" s="12"/>
     </row>
     <row r="3" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="53" t="s">
+      <c r="C3" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="53" t="s">
+      <c r="D3" s="46" t="s">
         <v>196</v>
       </c>
-      <c r="E3" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="53" t="s">
+      <c r="E3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="53" t="s">
+      <c r="G3" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="53" t="s">
+      <c r="H3" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I3" s="53"/>
-      <c r="J3" s="53" t="s">
+      <c r="I3" s="46"/>
+      <c r="J3" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K3" s="53" t="s">
+      <c r="K3" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="53" t="s">
+      <c r="L3" s="46" t="s">
         <v>188</v>
       </c>
-      <c r="M3" s="53" t="s">
+      <c r="M3" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O3" s="12"/>
@@ -11056,41 +11056,41 @@
       <c r="AA3" s="12"/>
     </row>
     <row r="4" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="53" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="53" t="s">
+      <c r="B4" s="46" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="53" t="s">
+      <c r="D4" s="46" t="s">
         <v>197</v>
       </c>
-      <c r="E4" s="53" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="53" t="s">
+      <c r="E4" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="53" t="s">
+      <c r="G4" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="53" t="s">
-        <v>38</v>
-      </c>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53" t="s">
+      <c r="H4" s="46" t="s">
+        <v>194</v>
+      </c>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K4" s="53" t="s">
+      <c r="K4" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="53" t="s">
-        <v>189</v>
-      </c>
-      <c r="M4" s="53" t="s">
+      <c r="L4" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="M4" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O4" s="12"/>
@@ -11108,41 +11108,41 @@
       <c r="AA4" s="12"/>
     </row>
     <row r="5" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="53" t="s">
+      <c r="A5" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="53" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="53" t="s">
+      <c r="B5" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="53" t="s">
+      <c r="D5" s="46" t="s">
         <v>198</v>
       </c>
-      <c r="E5" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" s="53" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="53" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5" s="53" t="s">
+      <c r="E5" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="G5" s="46" t="s">
+        <v>200</v>
+      </c>
+      <c r="H5" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53" t="s">
+      <c r="I5" s="46"/>
+      <c r="J5" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K5" s="53" t="s">
+      <c r="K5" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L5" s="53" t="s">
-        <v>190</v>
-      </c>
-      <c r="M5" s="53" t="s">
+      <c r="L5" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="M5" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O5" s="12"/>
@@ -11160,41 +11160,41 @@
       <c r="AA5" s="12"/>
     </row>
     <row r="6" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="53" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="53" t="s">
+      <c r="B6" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="53" t="s">
+      <c r="D6" s="46" t="s">
+        <v>201</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="E6" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="53" t="s">
+      <c r="G6" s="46" t="s">
         <v>200</v>
       </c>
-      <c r="G6" s="53" t="s">
-        <v>201</v>
-      </c>
-      <c r="H6" s="53" t="s">
+      <c r="H6" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53" t="s">
+      <c r="I6" s="46"/>
+      <c r="J6" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K6" s="53" t="s">
+      <c r="K6" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="53" t="s">
-        <v>191</v>
-      </c>
-      <c r="M6" s="53" t="s">
+      <c r="L6" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="M6" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O6" s="12"/>
@@ -11212,41 +11212,41 @@
       <c r="AA6" s="12"/>
     </row>
     <row r="7" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="53" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="53" t="s">
+      <c r="B7" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="46" t="s">
         <v>202</v>
       </c>
-      <c r="E7" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="53" t="s">
+      <c r="E7" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="F7" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="G7" s="46" t="s">
         <v>200</v>
       </c>
-      <c r="G7" s="53" t="s">
-        <v>201</v>
-      </c>
-      <c r="H7" s="53" t="s">
+      <c r="H7" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53" t="s">
+      <c r="I7" s="46"/>
+      <c r="J7" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K7" s="53" t="s">
+      <c r="K7" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="53" t="s">
-        <v>187</v>
-      </c>
-      <c r="M7" s="53" t="s">
+      <c r="L7" s="46" t="s">
+        <v>188</v>
+      </c>
+      <c r="M7" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O7" s="12"/>
@@ -11264,41 +11264,41 @@
       <c r="AA7" s="12"/>
     </row>
     <row r="8" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="53" t="s">
+      <c r="A8" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="53" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="53" t="s">
+      <c r="B8" s="46" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="53" t="s">
+      <c r="D8" s="46" t="s">
         <v>203</v>
       </c>
-      <c r="E8" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="53" t="s">
+      <c r="E8" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="G8" s="46" t="s">
         <v>200</v>
       </c>
-      <c r="G8" s="53" t="s">
-        <v>201</v>
-      </c>
-      <c r="H8" s="53" t="s">
+      <c r="H8" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53" t="s">
+      <c r="I8" s="46"/>
+      <c r="J8" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="53" t="s">
+      <c r="K8" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="53" t="s">
-        <v>188</v>
-      </c>
-      <c r="M8" s="53" t="s">
+      <c r="L8" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="M8" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O8" s="12"/>
@@ -11316,41 +11316,41 @@
       <c r="AA8" s="12"/>
     </row>
     <row r="9" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="53" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" s="53" t="s">
+      <c r="A9" s="46" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="53" t="s">
+      <c r="D9" s="46" t="s">
         <v>204</v>
       </c>
-      <c r="E9" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="G9" s="53" t="s">
-        <v>201</v>
-      </c>
-      <c r="H9" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53" t="s">
+      <c r="E9" s="46" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G9" s="46" t="s">
+        <v>206</v>
+      </c>
+      <c r="H9" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I9" s="46"/>
+      <c r="J9" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K9" s="53" t="s">
+      <c r="K9" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L9" s="53" t="s">
-        <v>191</v>
-      </c>
-      <c r="M9" s="53" t="s">
+      <c r="L9" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="M9" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O9" s="12"/>
@@ -11368,41 +11368,41 @@
       <c r="AA9" s="12"/>
     </row>
     <row r="10" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="53" t="s">
+      <c r="A10" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="53" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="53" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="53" t="s">
+      <c r="B10" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" s="46" t="s">
         <v>205</v>
       </c>
-      <c r="E10" s="53" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G10" s="53" t="s">
+      <c r="G10" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="H10" s="46" t="s">
         <v>207</v>
       </c>
-      <c r="H10" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I10" s="53"/>
-      <c r="J10" s="53" t="s">
+      <c r="I10" s="46"/>
+      <c r="J10" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K10" s="53" t="s">
+      <c r="K10" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="53" t="s">
+      <c r="L10" s="46" t="s">
         <v>187</v>
       </c>
-      <c r="M10" s="53" t="s">
+      <c r="M10" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O10" s="12"/>
@@ -11420,41 +11420,41 @@
       <c r="AA10" s="12"/>
     </row>
     <row r="11" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="53" t="s">
+      <c r="A11" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="53" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D11" s="53" t="s">
+      <c r="B11" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>211</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G11" s="46" t="s">
         <v>210</v>
       </c>
-      <c r="E11" s="53" t="s">
-        <v>73</v>
-      </c>
-      <c r="F11" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G11" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="H11" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I11" s="53"/>
-      <c r="J11" s="53" t="s">
+      <c r="H11" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I11" s="46"/>
+      <c r="J11" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K11" s="53" t="s">
+      <c r="K11" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="53" t="s">
-        <v>187</v>
-      </c>
-      <c r="M11" s="53" t="s">
+      <c r="L11" s="46" t="s">
+        <v>188</v>
+      </c>
+      <c r="M11" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O11" s="12"/>
@@ -11472,41 +11472,41 @@
       <c r="AA11" s="12"/>
     </row>
     <row r="12" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B12" s="53" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D12" s="53" t="s">
+      <c r="B12" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="46" t="s">
         <v>212</v>
       </c>
-      <c r="E12" s="53" t="s">
-        <v>74</v>
-      </c>
-      <c r="F12" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G12" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="H12" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I12" s="53"/>
-      <c r="J12" s="53" t="s">
+      <c r="D12" s="46" t="s">
+        <v>213</v>
+      </c>
+      <c r="E12" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="H12" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I12" s="46"/>
+      <c r="J12" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K12" s="53" t="s">
+      <c r="K12" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="53" t="s">
-        <v>188</v>
-      </c>
-      <c r="M12" s="53" t="s">
+      <c r="L12" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="M12" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O12" s="12"/>
@@ -11524,41 +11524,41 @@
       <c r="AA12" s="12"/>
     </row>
     <row r="13" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="53" t="s">
+      <c r="A13" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="53" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="53" t="s">
-        <v>213</v>
-      </c>
-      <c r="D13" s="53" t="s">
+      <c r="B13" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>215</v>
+      </c>
+      <c r="E13" s="46" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G13" s="46" t="s">
         <v>214</v>
       </c>
-      <c r="E13" s="53" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G13" s="53" t="s">
-        <v>215</v>
-      </c>
-      <c r="H13" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I13" s="53"/>
-      <c r="J13" s="53" t="s">
+      <c r="H13" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I13" s="46"/>
+      <c r="J13" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K13" s="53" t="s">
+      <c r="K13" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L13" s="53" t="s">
-        <v>190</v>
-      </c>
-      <c r="M13" s="53" t="s">
+      <c r="L13" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="M13" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O13" s="12"/>
@@ -11576,41 +11576,41 @@
       <c r="AA13" s="12"/>
     </row>
     <row r="14" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="53" t="s">
+      <c r="A14" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B14" s="53" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="53" t="s">
-        <v>213</v>
-      </c>
-      <c r="D14" s="53" t="s">
+      <c r="B14" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D14" s="46" t="s">
         <v>216</v>
       </c>
-      <c r="E14" s="53" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G14" s="53" t="s">
-        <v>215</v>
-      </c>
-      <c r="H14" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I14" s="53"/>
-      <c r="J14" s="53" t="s">
+      <c r="E14" s="46" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G14" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="H14" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K14" s="53" t="s">
+      <c r="K14" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L14" s="53" t="s">
-        <v>191</v>
-      </c>
-      <c r="M14" s="53" t="s">
+      <c r="L14" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="M14" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O14" s="12"/>
@@ -11628,41 +11628,41 @@
       <c r="AA14" s="12"/>
     </row>
     <row r="15" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53" t="s">
+      <c r="A15" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="53" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D15" s="53" t="s">
+      <c r="B15" s="46" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D15" s="46" t="s">
         <v>217</v>
       </c>
-      <c r="E15" s="53" t="s">
-        <v>81</v>
-      </c>
-      <c r="F15" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G15" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="H15" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I15" s="53"/>
-      <c r="J15" s="53" t="s">
+      <c r="E15" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G15" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="H15" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I15" s="46"/>
+      <c r="J15" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K15" s="53" t="s">
+      <c r="K15" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="53" t="s">
-        <v>187</v>
-      </c>
-      <c r="M15" s="53" t="s">
+      <c r="L15" s="46" t="s">
+        <v>188</v>
+      </c>
+      <c r="M15" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O15" s="12"/>
@@ -11680,41 +11680,41 @@
       <c r="AA15" s="12"/>
     </row>
     <row r="16" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="53" t="s">
+      <c r="A16" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="53" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D16" s="53" t="s">
+      <c r="B16" s="46" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16" s="46" t="s">
         <v>218</v>
       </c>
-      <c r="E16" s="53" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G16" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="H16" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I16" s="53"/>
-      <c r="J16" s="53" t="s">
+      <c r="E16" s="46" t="s">
+        <v>88</v>
+      </c>
+      <c r="F16" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G16" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="H16" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I16" s="46"/>
+      <c r="J16" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K16" s="53" t="s">
+      <c r="K16" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L16" s="53" t="s">
-        <v>188</v>
-      </c>
-      <c r="M16" s="53" t="s">
+      <c r="L16" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="M16" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O16" s="12"/>
@@ -11732,41 +11732,41 @@
       <c r="AA16" s="12"/>
     </row>
     <row r="17" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="53" t="s">
+      <c r="A17" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="53" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D17" s="53" t="s">
+      <c r="B17" s="46" t="s">
+        <v>95</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D17" s="46" t="s">
         <v>219</v>
       </c>
-      <c r="E17" s="53" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G17" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="H17" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I17" s="53"/>
-      <c r="J17" s="53" t="s">
+      <c r="E17" s="46" t="s">
+        <v>93</v>
+      </c>
+      <c r="F17" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G17" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="H17" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I17" s="46"/>
+      <c r="J17" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K17" s="53" t="s">
+      <c r="K17" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L17" s="53" t="s">
-        <v>189</v>
-      </c>
-      <c r="M17" s="53" t="s">
+      <c r="L17" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="M17" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O17" s="12"/>
@@ -11784,41 +11784,41 @@
       <c r="AA17" s="12"/>
     </row>
     <row r="18" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="53" t="s">
+      <c r="A18" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B18" s="53" t="s">
-        <v>95</v>
-      </c>
-      <c r="C18" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D18" s="53" t="s">
+      <c r="B18" s="46" t="s">
+        <v>183</v>
+      </c>
+      <c r="C18" s="46" t="s">
         <v>220</v>
       </c>
-      <c r="E18" s="53" t="s">
-        <v>93</v>
-      </c>
-      <c r="F18" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G18" s="53" t="s">
-        <v>211</v>
-      </c>
-      <c r="H18" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I18" s="53"/>
-      <c r="J18" s="53" t="s">
+      <c r="D18" s="46" t="s">
+        <v>221</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="F18" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>222</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="I18" s="46"/>
+      <c r="J18" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K18" s="53" t="s">
+      <c r="K18" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L18" s="53" t="s">
-        <v>190</v>
-      </c>
-      <c r="M18" s="53" t="s">
+      <c r="L18" s="46" t="s">
+        <v>188</v>
+      </c>
+      <c r="M18" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O18" s="12"/>
@@ -11836,41 +11836,41 @@
       <c r="AA18" s="12"/>
     </row>
     <row r="19" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="53" t="s">
+      <c r="A19" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B19" s="53" t="s">
-        <v>183</v>
-      </c>
-      <c r="C19" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="D19" s="53" t="s">
+      <c r="B19" s="46" t="s">
+        <v>184</v>
+      </c>
+      <c r="C19" s="46" t="s">
+        <v>220</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>223</v>
+      </c>
+      <c r="E19" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G19" s="46" t="s">
         <v>222</v>
       </c>
-      <c r="E19" s="53" t="s">
-        <v>99</v>
-      </c>
-      <c r="F19" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G19" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="H19" s="53" t="s">
-        <v>38</v>
-      </c>
-      <c r="I19" s="53"/>
-      <c r="J19" s="53" t="s">
+      <c r="H19" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K19" s="53" t="s">
+      <c r="K19" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L19" s="53" t="s">
-        <v>188</v>
-      </c>
-      <c r="M19" s="53" t="s">
+      <c r="L19" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="M19" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O19" s="12"/>
@@ -11888,41 +11888,41 @@
       <c r="AA19" s="12"/>
     </row>
     <row r="20" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="53" t="s">
+      <c r="A20" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C20" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="D20" s="53" t="s">
+      <c r="B20" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="C20" s="46" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="46" t="s">
         <v>224</v>
       </c>
-      <c r="E20" s="53" t="s">
-        <v>103</v>
-      </c>
-      <c r="F20" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G20" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="H20" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I20" s="53"/>
-      <c r="J20" s="53" t="s">
+      <c r="E20" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F20" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G20" s="46" t="s">
+        <v>222</v>
+      </c>
+      <c r="H20" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I20" s="46"/>
+      <c r="J20" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K20" s="53" t="s">
+      <c r="K20" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L20" s="53" t="s">
-        <v>189</v>
-      </c>
-      <c r="M20" s="53" t="s">
+      <c r="L20" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="M20" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O20" s="12"/>
@@ -11940,41 +11940,41 @@
       <c r="AA20" s="12"/>
     </row>
     <row r="21" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="53" t="s">
+      <c r="A21" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="C21" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="D21" s="53" t="s">
+      <c r="B21" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="C21" s="46" t="s">
+        <v>220</v>
+      </c>
+      <c r="D21" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E21" s="53" t="s">
-        <v>106</v>
-      </c>
-      <c r="F21" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G21" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="H21" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I21" s="53"/>
-      <c r="J21" s="53" t="s">
+      <c r="E21" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="F21" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="G21" s="46" t="s">
+        <v>222</v>
+      </c>
+      <c r="H21" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K21" s="53" t="s">
+      <c r="K21" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L21" s="53" t="s">
-        <v>190</v>
-      </c>
-      <c r="M21" s="53" t="s">
+      <c r="L21" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="M21" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O21" s="12"/>
@@ -11992,41 +11992,41 @@
       <c r="AA21" s="12"/>
     </row>
     <row r="22" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="53" t="s">
-        <v>86</v>
-      </c>
-      <c r="B22" s="53" t="s">
-        <v>186</v>
-      </c>
-      <c r="C22" s="53" t="s">
-        <v>221</v>
-      </c>
-      <c r="D22" s="53" t="s">
+      <c r="A22" s="46" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="46" t="s">
+        <v>212</v>
+      </c>
+      <c r="D22" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E22" s="53" t="s">
-        <v>110</v>
-      </c>
-      <c r="F22" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="G22" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="H22" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I22" s="53"/>
-      <c r="J22" s="53" t="s">
+      <c r="E22" s="46" t="s">
+        <v>116</v>
+      </c>
+      <c r="F22" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="G22" s="46" t="s">
+        <v>228</v>
+      </c>
+      <c r="H22" s="46" t="s">
+        <v>194</v>
+      </c>
+      <c r="I22" s="46"/>
+      <c r="J22" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K22" s="53" t="s">
+      <c r="K22" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L22" s="53" t="s">
-        <v>191</v>
-      </c>
-      <c r="M22" s="53" t="s">
+      <c r="L22" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="M22" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O22" s="12"/>
@@ -12044,41 +12044,41 @@
       <c r="AA22" s="12"/>
     </row>
     <row r="23" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="53" t="s">
+      <c r="A23" s="46" t="s">
         <v>119</v>
       </c>
-      <c r="B23" s="53" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" s="53" t="s">
-        <v>213</v>
-      </c>
-      <c r="D23" s="53" t="s">
+      <c r="B23" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="46" t="s">
+        <v>208</v>
+      </c>
+      <c r="D23" s="46" t="s">
+        <v>229</v>
+      </c>
+      <c r="E23" s="46" t="s">
+        <v>120</v>
+      </c>
+      <c r="F23" s="46" t="s">
         <v>227</v>
       </c>
-      <c r="E23" s="53" t="s">
-        <v>116</v>
-      </c>
-      <c r="F23" s="53" t="s">
+      <c r="G23" s="46" t="s">
         <v>228</v>
       </c>
-      <c r="G23" s="53" t="s">
-        <v>229</v>
-      </c>
-      <c r="H23" s="53" t="s">
-        <v>194</v>
-      </c>
-      <c r="I23" s="53"/>
-      <c r="J23" s="53" t="s">
+      <c r="H23" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K23" s="53" t="s">
+      <c r="K23" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L23" s="53" t="s">
-        <v>187</v>
-      </c>
-      <c r="M23" s="53" t="s">
+      <c r="L23" s="46" t="s">
+        <v>188</v>
+      </c>
+      <c r="M23" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O23" s="12"/>
@@ -12096,41 +12096,41 @@
       <c r="AA23" s="12"/>
     </row>
     <row r="24" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="53" t="s">
-        <v>119</v>
-      </c>
-      <c r="B24" s="53" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="D24" s="53" t="s">
+      <c r="A24" s="46" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24" s="46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="46" t="s">
         <v>230</v>
       </c>
-      <c r="E24" s="53" t="s">
-        <v>120</v>
-      </c>
-      <c r="F24" s="53" t="s">
-        <v>228</v>
-      </c>
-      <c r="G24" s="53" t="s">
-        <v>229</v>
-      </c>
-      <c r="H24" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="I24" s="53"/>
-      <c r="J24" s="53" t="s">
+      <c r="E24" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="F24" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="G24" s="46" t="s">
+        <v>232</v>
+      </c>
+      <c r="H24" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="I24" s="46"/>
+      <c r="J24" s="46" t="s">
         <v>195</v>
       </c>
-      <c r="K24" s="53" t="s">
+      <c r="K24" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="L24" s="53" t="s">
-        <v>188</v>
-      </c>
-      <c r="M24" s="53" t="s">
+      <c r="L24" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="M24" s="46" t="s">
         <v>192</v>
       </c>
       <c r="O24" s="12"/>
@@ -12147,44 +12147,21 @@
       <c r="Z24" s="12"/>
       <c r="AA24" s="12"/>
     </row>
-    <row r="25" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53" t="s">
-        <v>123</v>
-      </c>
-      <c r="B25" s="53" t="s">
-        <v>14</v>
-      </c>
-      <c r="C25" s="53" t="s">
-        <v>34</v>
-      </c>
-      <c r="D25" s="53" t="s">
-        <v>231</v>
-      </c>
-      <c r="E25" s="53" t="s">
-        <v>128</v>
-      </c>
-      <c r="F25" s="53" t="s">
-        <v>232</v>
-      </c>
-      <c r="G25" s="53" t="s">
-        <v>233</v>
-      </c>
-      <c r="H25" s="53" t="s">
-        <v>38</v>
-      </c>
-      <c r="I25" s="53"/>
-      <c r="J25" s="53" t="s">
-        <v>195</v>
-      </c>
-      <c r="K25" s="53" t="s">
-        <v>22</v>
-      </c>
-      <c r="L25" s="53" t="s">
-        <v>189</v>
-      </c>
-      <c r="M25" s="53" t="s">
-        <v>192</v>
-      </c>
+    <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
       <c r="O25" s="12"/>
       <c r="P25" s="12"/>
       <c r="Q25" s="12"/>
@@ -17826,33 +17803,7 @@
       <c r="AA219" s="12"/>
     </row>
     <row r="220" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A220" s="12"/>
-      <c r="B220" s="12"/>
-      <c r="C220" s="12"/>
-      <c r="D220" s="12"/>
-      <c r="E220" s="12"/>
-      <c r="F220" s="12"/>
-      <c r="G220" s="12"/>
-      <c r="H220" s="12"/>
-      <c r="I220" s="12"/>
-      <c r="J220" s="12"/>
-      <c r="K220" s="12"/>
-      <c r="L220" s="12"/>
-      <c r="M220" s="12"/>
-      <c r="N220" s="12"/>
-      <c r="O220" s="12"/>
-      <c r="P220" s="12"/>
-      <c r="Q220" s="12"/>
-      <c r="R220" s="12"/>
-      <c r="S220" s="12"/>
-      <c r="T220" s="12"/>
-      <c r="U220" s="12"/>
-      <c r="V220" s="12"/>
-      <c r="W220" s="12"/>
-      <c r="X220" s="12"/>
-      <c r="Y220" s="12"/>
-      <c r="Z220" s="12"/>
-      <c r="AA220" s="12"/>
+      <c r="I220" s="13"/>
     </row>
     <row r="221" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I221" s="13"/>
@@ -20191,21 +20142,18 @@
     <row r="999" spans="9:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I999" s="13"/>
     </row>
-    <row r="1000" spans="9:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I1000" s="13"/>
-    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2:K5" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2:K4" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Pass,Fail,Re-open"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I1:I1000" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I1:I999" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Allocated To"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H5" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H4" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J2:J5" xr:uid="{00000000-0002-0000-0200-000003000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J2:J4" xr:uid="{00000000-0002-0000-0200-000003000000}">
       <formula1>"Completed,Pendig,Not a Bug,Defferd"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>